<commit_message>
chore: push latest changes to production (Nuntec proxy fix and UI updates)
</commit_message>
<xml_diff>
--- a/solicitacao_711_itens.xlsx
+++ b/solicitacao_711_itens.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://agropecuarianadiana-my.sharepoint.com/personal/bruno_siqueira_nadiana_com_br/Documents/Área de Trabalho/Projetos/Sistema Nadiana/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_C9470121D0B0FA4D3A60024B9816B11DA02D209F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C85220FB-55C1-4541-80C2-5B68F6EE8DF2}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_C9470121D0B0FA4D3A60024B9816B11DA02D209F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9FD2BDD-8313-41BE-B290-5796C06AF362}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Itens Solicitação #711" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Itens Solicitação #711'!$A$1:$H$1</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -1390,17 +1393,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1757,7 +1750,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H219"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.796875" customWidth="1"/>
     <col min="2" max="2" width="15.796875" customWidth="1"/>
@@ -1769,7 +1762,7 @@
     <col min="8" max="8" width="20.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1795,7 +1788,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1815,7 +1808,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1835,7 +1828,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1855,7 +1848,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1875,7 +1868,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1895,7 +1888,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1915,7 +1908,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1935,7 +1928,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1955,7 +1948,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1975,7 +1968,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1995,7 +1988,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2015,7 +2008,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2035,7 +2028,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2055,7 +2048,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -2075,7 +2068,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2095,7 +2088,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -2115,7 +2108,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -2135,7 +2128,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2155,7 +2148,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -2175,7 +2168,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -2195,7 +2188,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -2215,7 +2208,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -2235,7 +2228,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -2255,7 +2248,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -2275,7 +2268,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -2295,7 +2288,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -2315,7 +2308,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2335,7 +2328,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -2355,7 +2348,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -2375,7 +2368,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -2395,7 +2388,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -2415,7 +2408,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -2435,7 +2428,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -2455,7 +2448,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -2475,7 +2468,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -2495,7 +2488,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -2515,7 +2508,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
@@ -2535,7 +2528,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
@@ -2555,7 +2548,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
@@ -2575,7 +2568,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
@@ -2595,7 +2588,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>41</v>
       </c>
@@ -2615,7 +2608,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>42</v>
       </c>
@@ -2635,7 +2628,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
@@ -2655,7 +2648,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -2675,7 +2668,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -2695,7 +2688,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -2715,7 +2708,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="48" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
@@ -2735,7 +2728,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="49" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -2755,7 +2748,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="50" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>49</v>
       </c>
@@ -2775,7 +2768,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>50</v>
       </c>
@@ -2795,7 +2788,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="52" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>51</v>
       </c>
@@ -2815,7 +2808,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="53" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>52</v>
       </c>
@@ -2835,7 +2828,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="54" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>53</v>
       </c>
@@ -2855,7 +2848,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="55" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>54</v>
       </c>
@@ -2875,7 +2868,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="56" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>55</v>
       </c>
@@ -2895,7 +2888,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="57" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>56</v>
       </c>
@@ -2915,7 +2908,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="58" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>57</v>
       </c>
@@ -2935,7 +2928,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="59" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>58</v>
       </c>
@@ -2955,7 +2948,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="60" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>59</v>
       </c>
@@ -2975,7 +2968,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="61" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>60</v>
       </c>
@@ -2995,7 +2988,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="62" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>61</v>
       </c>
@@ -3015,7 +3008,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="63" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>62</v>
       </c>
@@ -3035,7 +3028,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="64" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>63</v>
       </c>
@@ -3055,7 +3048,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="65" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>64</v>
       </c>
@@ -3075,7 +3068,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="66" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>65</v>
       </c>
@@ -3095,7 +3088,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="67" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>66</v>
       </c>
@@ -3115,7 +3108,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="68" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>67</v>
       </c>
@@ -3135,7 +3128,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="69" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>68</v>
       </c>
@@ -3155,7 +3148,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="70" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>69</v>
       </c>
@@ -3175,7 +3168,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="71" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>70</v>
       </c>
@@ -3195,7 +3188,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="72" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>71</v>
       </c>
@@ -3215,7 +3208,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="73" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>72</v>
       </c>
@@ -3235,7 +3228,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="74" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>73</v>
       </c>
@@ -3255,7 +3248,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="75" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>74</v>
       </c>
@@ -3275,7 +3268,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="76" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>75</v>
       </c>
@@ -3295,7 +3288,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="77" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>76</v>
       </c>
@@ -3315,7 +3308,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="78" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>77</v>
       </c>
@@ -3335,7 +3328,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="79" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>78</v>
       </c>
@@ -3355,7 +3348,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="80" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>79</v>
       </c>
@@ -3375,7 +3368,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="81" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>80</v>
       </c>
@@ -3395,7 +3388,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="82" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>81</v>
       </c>
@@ -3415,7 +3408,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="83" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>82</v>
       </c>
@@ -3435,7 +3428,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="84" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>83</v>
       </c>
@@ -3455,7 +3448,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="85" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>84</v>
       </c>
@@ -3475,7 +3468,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="86" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>85</v>
       </c>
@@ -3495,7 +3488,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="87" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>86</v>
       </c>
@@ -3515,7 +3508,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="88" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>87</v>
       </c>
@@ -3535,7 +3528,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="89" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>88</v>
       </c>
@@ -3555,7 +3548,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="90" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>89</v>
       </c>
@@ -3575,7 +3568,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="91" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>90</v>
       </c>
@@ -3595,7 +3588,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="92" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>91</v>
       </c>
@@ -3615,7 +3608,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="93" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>92</v>
       </c>
@@ -3635,7 +3628,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="94" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>93</v>
       </c>
@@ -3655,7 +3648,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="95" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>94</v>
       </c>
@@ -3675,7 +3668,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="96" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>95</v>
       </c>
@@ -3695,7 +3688,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="97" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>96</v>
       </c>
@@ -3715,7 +3708,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="98" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>97</v>
       </c>
@@ -3735,7 +3728,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="99" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>98</v>
       </c>
@@ -3755,7 +3748,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="100" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>99</v>
       </c>
@@ -3775,7 +3768,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="101" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>100</v>
       </c>
@@ -3795,7 +3788,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="102" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>101</v>
       </c>
@@ -3815,7 +3808,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="103" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>102</v>
       </c>
@@ -3835,7 +3828,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="104" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>103</v>
       </c>
@@ -3855,7 +3848,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="105" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>104</v>
       </c>
@@ -3875,7 +3868,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="106" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>105</v>
       </c>
@@ -3895,7 +3888,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="107" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>106</v>
       </c>
@@ -3915,7 +3908,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="108" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>107</v>
       </c>
@@ -3935,7 +3928,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="109" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>108</v>
       </c>
@@ -3955,7 +3948,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="110" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>109</v>
       </c>
@@ -3975,7 +3968,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="111" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>110</v>
       </c>
@@ -3995,7 +3988,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="112" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>111</v>
       </c>
@@ -4015,7 +4008,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="113" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>112</v>
       </c>
@@ -4035,7 +4028,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="114" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>113</v>
       </c>
@@ -4055,7 +4048,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="115" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>114</v>
       </c>
@@ -4075,7 +4068,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="116" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>115</v>
       </c>
@@ -4095,7 +4088,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="117" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>116</v>
       </c>
@@ -4115,7 +4108,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="118" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>117</v>
       </c>
@@ -4135,7 +4128,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="119" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>118</v>
       </c>
@@ -4155,7 +4148,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="120" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>119</v>
       </c>
@@ -4175,7 +4168,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="121" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>120</v>
       </c>
@@ -4195,7 +4188,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="122" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>121</v>
       </c>
@@ -4215,7 +4208,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="123" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>122</v>
       </c>
@@ -4235,7 +4228,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="124" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>123</v>
       </c>
@@ -4255,7 +4248,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="125" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>124</v>
       </c>
@@ -4275,7 +4268,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="126" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>125</v>
       </c>
@@ -4295,7 +4288,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="127" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>126</v>
       </c>
@@ -4315,7 +4308,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="128" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>127</v>
       </c>
@@ -4335,7 +4328,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="129" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>128</v>
       </c>
@@ -4355,7 +4348,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="130" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>129</v>
       </c>
@@ -4375,7 +4368,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="131" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>130</v>
       </c>
@@ -4395,7 +4388,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="132" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>131</v>
       </c>
@@ -4415,7 +4408,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="133" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>132</v>
       </c>
@@ -4435,7 +4428,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="134" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>133</v>
       </c>
@@ -4455,7 +4448,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="135" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>134</v>
       </c>
@@ -4475,7 +4468,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="136" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>135</v>
       </c>
@@ -4495,7 +4488,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="137" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>136</v>
       </c>
@@ -4515,7 +4508,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="138" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>137</v>
       </c>
@@ -4535,7 +4528,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="139" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>138</v>
       </c>
@@ -4555,7 +4548,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="140" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>139</v>
       </c>
@@ -4575,7 +4568,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="141" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>140</v>
       </c>
@@ -4595,7 +4588,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="142" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>141</v>
       </c>
@@ -4615,7 +4608,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="143" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>142</v>
       </c>
@@ -4635,7 +4628,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="144" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>143</v>
       </c>
@@ -4655,7 +4648,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="145" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A145">
         <v>144</v>
       </c>
@@ -4675,7 +4668,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="146" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>145</v>
       </c>
@@ -4695,7 +4688,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="147" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>146</v>
       </c>
@@ -4715,7 +4708,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="148" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>147</v>
       </c>
@@ -4735,7 +4728,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="149" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>148</v>
       </c>
@@ -4755,7 +4748,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="150" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>149</v>
       </c>
@@ -4775,7 +4768,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="151" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>150</v>
       </c>
@@ -4795,7 +4788,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="152" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>151</v>
       </c>
@@ -4815,7 +4808,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="153" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>152</v>
       </c>
@@ -4835,7 +4828,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="154" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>153</v>
       </c>
@@ -4855,7 +4848,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="155" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>154</v>
       </c>
@@ -4875,7 +4868,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="156" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>155</v>
       </c>
@@ -4895,7 +4888,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="157" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>156</v>
       </c>
@@ -4915,7 +4908,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="158" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>157</v>
       </c>
@@ -4935,7 +4928,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="159" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>158</v>
       </c>
@@ -4955,7 +4948,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="160" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>159</v>
       </c>
@@ -4975,7 +4968,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="161" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>160</v>
       </c>
@@ -4995,7 +4988,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="162" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>161</v>
       </c>
@@ -5015,7 +5008,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="163" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>162</v>
       </c>
@@ -5035,7 +5028,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="164" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>163</v>
       </c>
@@ -5055,7 +5048,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="165" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A165">
         <v>164</v>
       </c>
@@ -5075,7 +5068,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="166" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A166">
         <v>165</v>
       </c>
@@ -5095,7 +5088,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="167" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A167">
         <v>166</v>
       </c>
@@ -5115,7 +5108,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="168" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A168">
         <v>167</v>
       </c>
@@ -5135,7 +5128,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="169" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A169">
         <v>168</v>
       </c>
@@ -5155,7 +5148,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="170" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A170">
         <v>169</v>
       </c>
@@ -5175,7 +5168,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="171" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>170</v>
       </c>
@@ -5195,7 +5188,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="172" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A172">
         <v>171</v>
       </c>
@@ -5215,7 +5208,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="173" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A173">
         <v>172</v>
       </c>
@@ -5235,7 +5228,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="174" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>173</v>
       </c>
@@ -5255,7 +5248,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="175" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A175">
         <v>174</v>
       </c>
@@ -5275,7 +5268,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="176" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A176">
         <v>175</v>
       </c>
@@ -5295,7 +5288,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="177" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>176</v>
       </c>
@@ -5315,7 +5308,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="178" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>177</v>
       </c>
@@ -5335,7 +5328,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="179" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>178</v>
       </c>
@@ -5355,7 +5348,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="180" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>179</v>
       </c>
@@ -5375,7 +5368,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="181" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A181">
         <v>180</v>
       </c>
@@ -5395,7 +5388,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="182" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A182">
         <v>181</v>
       </c>
@@ -5415,7 +5408,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="183" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A183">
         <v>182</v>
       </c>
@@ -5435,7 +5428,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="184" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A184">
         <v>183</v>
       </c>
@@ -5455,7 +5448,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="185" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A185">
         <v>184</v>
       </c>
@@ -5475,7 +5468,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="186" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A186">
         <v>185</v>
       </c>
@@ -5495,7 +5488,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="187" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A187">
         <v>186</v>
       </c>
@@ -5515,7 +5508,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="188" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A188">
         <v>187</v>
       </c>
@@ -5535,7 +5528,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="189" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A189">
         <v>188</v>
       </c>
@@ -5555,7 +5548,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="190" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A190">
         <v>189</v>
       </c>
@@ -5575,7 +5568,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="191" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A191">
         <v>190</v>
       </c>
@@ -5595,7 +5588,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="192" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A192">
         <v>191</v>
       </c>
@@ -5615,7 +5608,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="193" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A193">
         <v>192</v>
       </c>
@@ -5635,7 +5628,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="194" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A194">
         <v>193</v>
       </c>
@@ -5655,7 +5648,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="195" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>194</v>
       </c>
@@ -5675,7 +5668,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="196" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A196">
         <v>195</v>
       </c>
@@ -5695,7 +5688,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="197" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A197">
         <v>196</v>
       </c>
@@ -5715,7 +5708,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="198" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A198">
         <v>197</v>
       </c>
@@ -5735,7 +5728,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="199" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A199">
         <v>198</v>
       </c>
@@ -5755,7 +5748,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="200" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A200">
         <v>199</v>
       </c>
@@ -5775,7 +5768,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="201" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A201">
         <v>200</v>
       </c>
@@ -5795,7 +5788,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="202" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A202">
         <v>201</v>
       </c>
@@ -5815,7 +5808,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="203" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A203">
         <v>202</v>
       </c>
@@ -5835,7 +5828,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="204" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A204">
         <v>203</v>
       </c>
@@ -5855,7 +5848,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="205" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A205">
         <v>204</v>
       </c>
@@ -5875,7 +5868,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="206" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A206">
         <v>205</v>
       </c>
@@ -5895,7 +5888,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="207" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A207">
         <v>206</v>
       </c>
@@ -5915,7 +5908,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="208" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A208">
         <v>207</v>
       </c>
@@ -5935,7 +5928,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="209" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A209">
         <v>208</v>
       </c>
@@ -5955,7 +5948,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="210" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A210">
         <v>209</v>
       </c>
@@ -5975,7 +5968,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="211" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A211">
         <v>210</v>
       </c>
@@ -5995,7 +5988,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="212" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A212">
         <v>211</v>
       </c>
@@ -6015,7 +6008,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="213" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A213">
         <v>212</v>
       </c>
@@ -6035,7 +6028,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="214" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A214">
         <v>213</v>
       </c>
@@ -6055,7 +6048,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="215" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A215">
         <v>214</v>
       </c>
@@ -6075,7 +6068,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="216" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A216">
         <v>215</v>
       </c>
@@ -6095,7 +6088,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="217" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A217">
         <v>216</v>
       </c>
@@ -6115,7 +6108,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="218" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A218">
         <v>217</v>
       </c>
@@ -6135,7 +6128,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="219" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A219">
         <v>218</v>
       </c>
@@ -6156,8 +6149,9 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="E1:E1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>

</xml_diff>